<commit_message>
Parse Android and iOS string files properly
Android `.xml` files are now parsed with lxml instead of regular
expressions, so strings with extra attributes (e.g.
`translatable="false"`) or that span multiple lines are no longer
skipped. `<plurals>` and `<string-array>` resources are skipped with a
warning.

iOS `.strings` files now support `/* */` comments, and `//` inside a
value (e.g. a URL) is no longer treated as a comment.

XML entities and the escape sequences of both formats are decoded when
reading and encoded when writing, so:

- Other file types contain the actual text (e.g. `I'm` instead of
  `I\'m`).
- Values with `&`, `<`, quotes or backslashes produce valid `.xml` and
  `.strings` files.

Strings with inline markup (e.g. `Hello <b>World</b>`) are kept
verbatim.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/files/template-with-comments/strings.xlsx
+++ b/tests/files/template-with-comments/strings.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -688,7 +688,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>I\'m happy to be here</t>
+          <t>I'm happy to be here</t>
         </is>
       </c>
     </row>
@@ -700,7 +700,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>C\'est comme ça</t>
+          <t>C'est comme ça</t>
         </is>
       </c>
     </row>

</xml_diff>